<commit_message>
Added chat history logging with SQLite
</commit_message>
<xml_diff>
--- a/chat_history_log.xlsx
+++ b/chat_history_log.xlsx
@@ -1,75 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bainandcompany-my.sharepoint.com/personal/abhay_singh2_bain_com/Documents/Documents/Python Scripts/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_2B59D2BFD3B05674E67EB313563088B35299F038" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D54C2E0-BAF6-4087-A676-E630CFACFF11}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>Timestamp</t>
-  </si>
-  <si>
-    <t>Question</t>
-  </si>
-  <si>
-    <t>Answer</t>
-  </si>
-  <si>
-    <t>Sources</t>
-  </si>
-  <si>
-    <t>2025-05-29 08:01:31</t>
-  </si>
-  <si>
-    <t>Bain CEO?</t>
-  </si>
-  <si>
-    <t>As of February 2022, the CEO of Bain &amp; Company is Manny Maceda. Please note that this may change over time, so it's advisable to verify from the official Bain &amp; Company website for the most current information. 
-Source:
-"Bain &amp; Company Leadership". Bain &amp; Company. Retrieved from: https://www.bain.com/about/leadership/</t>
-  </si>
-  <si>
-    <t>Bain Overview FAQ.pdf (page 5), Full RFP FAQ Export.pdf (page 3), Bain Overview FAQ.pdf (page 2), Bain Overview FAQ.pdf (page 1), Full RFP FAQ Export.pdf (page 7), GRI report 2023.pdf (page 7), GRI report 2023.pdf (page 32), Bain Overview FAQ.pdf (page 6), Bain Overview FAQ.pdf (page 4), Full RFP FAQ Export.pdf (page 8), GRI report 2023.pdf (page 25), bain-wef-and-tcfd-report-2023.pdf (page 2), Bain Overview FAQ.pdf (page 3), Full RFP FAQ Export.pdf (page 5), Bain Overview FAQ.pdf (page 7), bain-wef-and-tcfd-report-2023.pdf (page 10), Full RFP FAQ Export.pdf (page 9), bain-wef-and-tcfd-report-2023.pdf (page 8), sustainable-procurement-factsheet-v3-05.02.2024.pdf (page 1), Full RFP FAQ Export.pdf (page 6)</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -84,43 +46,93 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -408,41 +420,58 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="18.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="255.77734375" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Answer</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Sources</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2025-05-29 08:01:31</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Bain CEO?</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>As of February 2022, the CEO of Bain &amp; Company is Manny Maceda. Please note that this may change over time, so it's advisable to verify from the official Bain &amp; Company website for the most current information. 
+Source:
+"Bain &amp; Company Leadership". Bain &amp; Company. Retrieved from: https://www.bain.com/about/leadership/</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Bain Overview FAQ.pdf (page 5), Full RFP FAQ Export.pdf (page 3), Bain Overview FAQ.pdf (page 2), Bain Overview FAQ.pdf (page 1), Full RFP FAQ Export.pdf (page 7), GRI report 2023.pdf (page 7), GRI report 2023.pdf (page 32), Bain Overview FAQ.pdf (page 6), Bain Overview FAQ.pdf (page 4), Full RFP FAQ Export.pdf (page 8), GRI report 2023.pdf (page 25), bain-wef-and-tcfd-report-2023.pdf (page 2), Bain Overview FAQ.pdf (page 3), Full RFP FAQ Export.pdf (page 5), Bain Overview FAQ.pdf (page 7), bain-wef-and-tcfd-report-2023.pdf (page 10), Full RFP FAQ Export.pdf (page 9), bain-wef-and-tcfd-report-2023.pdf (page 8), sustainable-procurement-factsheet-v3-05.02.2024.pdf (page 1), Full RFP FAQ Export.pdf (page 6)</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>